<commit_message>
Fixed issue with one extrusion below the minimum Misumi hole spacing
</commit_message>
<xml_diff>
--- a/CAD/Voron_Cascade_BOM.xlsx
+++ b/CAD/Voron_Cascade_BOM.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="483">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="484">
   <si>
     <t>Section / Item</t>
   </si>
@@ -99,10 +99,10 @@
     <t>HFSB6-3060-500-TPW-Z8-XA350-XB380-YA15-YB485</t>
   </si>
   <si>
-    <t>2020, 235mm, both ends tapped, wrench access holes</t>
-  </si>
-  <si>
-    <t>HFSB5-2020-235-TPW-Z6-YA50-YB75-YC205-YD230</t>
+    <t>2020, 237mm, both ends tapped, wrench access holes</t>
+  </si>
+  <si>
+    <t>HFSB5-2020-237-TPW-AH50-BH75-CH205-DH230</t>
   </si>
   <si>
     <t>Working Enclosure Frame</t>
@@ -796,6 +796,9 @@
   </si>
   <si>
     <t>Loctite 242 or equivalent</t>
+  </si>
+  <si>
+    <t>1/4”x4” hardened steel dowel</t>
   </si>
   <si>
     <t>2mm x 100mm (4") zip ties</t>
@@ -2787,7 +2790,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T1041"/>
+  <dimension ref="A1:T1042"/>
   <sheetFormatPr defaultColWidth="12.6667" defaultRowHeight="15.75" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="50.5" style="1" customWidth="1"/>
@@ -8027,7 +8030,7 @@
       </c>
       <c r="B200" s="5"/>
       <c r="C200" s="7">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="D200" s="5"/>
       <c r="E200" s="5"/>
@@ -8053,7 +8056,7 @@
       </c>
       <c r="B201" s="5"/>
       <c r="C201" s="7">
-        <v>3</v>
+        <v>50</v>
       </c>
       <c r="D201" s="5"/>
       <c r="E201" s="5"/>
@@ -8079,7 +8082,7 @@
       </c>
       <c r="B202" s="5"/>
       <c r="C202" s="7">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="D202" s="5"/>
       <c r="E202" s="5"/>
@@ -8103,11 +8106,9 @@
       <c r="A203" t="s" s="6">
         <v>264</v>
       </c>
-      <c r="B203" t="s" s="6">
-        <v>265</v>
-      </c>
+      <c r="B203" s="5"/>
       <c r="C203" s="7">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="D203" s="5"/>
       <c r="E203" s="5"/>
@@ -8128,9 +8129,15 @@
       <c r="T203" s="5"/>
     </row>
     <row r="204" ht="13.65" customHeight="1">
-      <c r="A204" s="5"/>
-      <c r="B204" s="5"/>
-      <c r="C204" s="5"/>
+      <c r="A204" t="s" s="6">
+        <v>265</v>
+      </c>
+      <c r="B204" t="s" s="6">
+        <v>266</v>
+      </c>
+      <c r="C204" s="7">
+        <v>50</v>
+      </c>
       <c r="D204" s="5"/>
       <c r="E204" s="5"/>
       <c r="F204" s="5"/>
@@ -8150,12 +8157,8 @@
       <c r="T204" s="5"/>
     </row>
     <row r="205" ht="13.65" customHeight="1">
-      <c r="A205" t="s" s="4">
-        <v>266</v>
-      </c>
-      <c r="B205" t="s" s="6">
-        <v>267</v>
-      </c>
+      <c r="A205" s="5"/>
+      <c r="B205" s="5"/>
       <c r="C205" s="5"/>
       <c r="D205" s="5"/>
       <c r="E205" s="5"/>
@@ -8176,13 +8179,13 @@
       <c r="T205" s="5"/>
     </row>
     <row r="206" ht="13.65" customHeight="1">
-      <c r="A206" t="s" s="6">
+      <c r="A206" t="s" s="4">
+        <v>267</v>
+      </c>
+      <c r="B206" t="s" s="6">
         <v>268</v>
       </c>
-      <c r="B206" s="5"/>
-      <c r="C206" s="7">
-        <v>1</v>
-      </c>
+      <c r="C206" s="5"/>
       <c r="D206" s="5"/>
       <c r="E206" s="5"/>
       <c r="F206" s="5"/>
@@ -8228,9 +8231,13 @@
       <c r="T207" s="5"/>
     </row>
     <row r="208" ht="13.65" customHeight="1">
-      <c r="A208" s="5"/>
+      <c r="A208" t="s" s="6">
+        <v>270</v>
+      </c>
       <c r="B208" s="5"/>
-      <c r="C208" s="5"/>
+      <c r="C208" s="7">
+        <v>1</v>
+      </c>
       <c r="D208" s="5"/>
       <c r="E208" s="5"/>
       <c r="F208" s="5"/>
@@ -8250,12 +8257,8 @@
       <c r="T208" s="5"/>
     </row>
     <row r="209" ht="13.65" customHeight="1">
-      <c r="A209" t="s" s="4">
-        <v>270</v>
-      </c>
-      <c r="B209" t="s" s="6">
-        <v>271</v>
-      </c>
+      <c r="A209" s="5"/>
+      <c r="B209" s="5"/>
       <c r="C209" s="5"/>
       <c r="D209" s="5"/>
       <c r="E209" s="5"/>
@@ -8276,13 +8279,13 @@
       <c r="T209" s="5"/>
     </row>
     <row r="210" ht="13.65" customHeight="1">
-      <c r="A210" t="s" s="6">
+      <c r="A210" t="s" s="4">
+        <v>271</v>
+      </c>
+      <c r="B210" t="s" s="6">
         <v>272</v>
       </c>
-      <c r="B210" s="5"/>
-      <c r="C210" s="7">
-        <v>1</v>
-      </c>
+      <c r="C210" s="5"/>
       <c r="D210" s="5"/>
       <c r="E210" s="5"/>
       <c r="F210" s="5"/>
@@ -8383,10 +8386,10 @@
       <c r="A214" t="s" s="6">
         <v>276</v>
       </c>
-      <c r="B214" t="s" s="6">
-        <v>277</v>
-      </c>
-      <c r="C214" s="5"/>
+      <c r="B214" s="5"/>
+      <c r="C214" s="7">
+        <v>1</v>
+      </c>
       <c r="D214" s="5"/>
       <c r="E214" s="5"/>
       <c r="F214" s="5"/>
@@ -8407,12 +8410,12 @@
     </row>
     <row r="215" ht="13.65" customHeight="1">
       <c r="A215" t="s" s="6">
+        <v>277</v>
+      </c>
+      <c r="B215" t="s" s="6">
         <v>278</v>
       </c>
-      <c r="B215" s="5"/>
-      <c r="C215" s="7">
-        <v>1</v>
-      </c>
+      <c r="C215" s="5"/>
       <c r="D215" s="5"/>
       <c r="E215" s="5"/>
       <c r="F215" s="5"/>
@@ -8510,9 +8513,13 @@
       <c r="T218" s="5"/>
     </row>
     <row r="219" ht="13.65" customHeight="1">
-      <c r="A219" s="5"/>
+      <c r="A219" t="s" s="6">
+        <v>282</v>
+      </c>
       <c r="B219" s="5"/>
-      <c r="C219" s="5"/>
+      <c r="C219" s="7">
+        <v>1</v>
+      </c>
       <c r="D219" s="5"/>
       <c r="E219" s="5"/>
       <c r="F219" s="5"/>
@@ -26614,6 +26621,28 @@
       <c r="R1041" s="5"/>
       <c r="S1041" s="5"/>
       <c r="T1041" s="5"/>
+    </row>
+    <row r="1042" ht="13.65" customHeight="1">
+      <c r="A1042" s="5"/>
+      <c r="B1042" s="5"/>
+      <c r="C1042" s="5"/>
+      <c r="D1042" s="5"/>
+      <c r="E1042" s="5"/>
+      <c r="F1042" s="5"/>
+      <c r="G1042" s="5"/>
+      <c r="H1042" s="5"/>
+      <c r="I1042" s="5"/>
+      <c r="J1042" s="5"/>
+      <c r="K1042" s="5"/>
+      <c r="L1042" s="5"/>
+      <c r="M1042" s="5"/>
+      <c r="N1042" s="5"/>
+      <c r="O1042" s="5"/>
+      <c r="P1042" s="5"/>
+      <c r="Q1042" s="5"/>
+      <c r="R1042" s="5"/>
+      <c r="S1042" s="5"/>
+      <c r="T1042" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
@@ -26644,7 +26673,7 @@
   <sheetData>
     <row r="1" ht="13.65" customHeight="1">
       <c r="A1" t="s" s="2">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -26655,130 +26684,130 @@
     </row>
     <row r="2" ht="13.65" customHeight="1">
       <c r="A2" t="s" s="12">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B2" t="s" s="12">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C2" t="s" s="12">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D2" t="s" s="12">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E2" t="s" s="12">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F2" t="s" s="12">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="G2" s="5"/>
     </row>
     <row r="3" ht="13.65" customHeight="1">
       <c r="A3" t="s" s="6">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B3" t="s" s="6">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C3" s="7">
         <v>1</v>
       </c>
       <c r="D3" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E3" t="s" s="6">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F3" t="s" s="6">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="G3" t="s" s="13">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="4" ht="13.65" customHeight="1">
       <c r="A4" s="5"/>
       <c r="B4" t="s" s="6">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C4" s="7">
         <v>1</v>
       </c>
       <c r="D4" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E4" t="s" s="6">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F4" t="s" s="14">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="G4" t="s" s="15">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="5" ht="13.65" customHeight="1">
       <c r="A5" s="5"/>
       <c r="B5" t="s" s="6">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C5" s="7">
         <v>1</v>
       </c>
       <c r="D5" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E5" t="s" s="6">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F5" t="s" s="14">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="G5" t="s" s="15">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="6" ht="13.65" customHeight="1">
       <c r="A6" s="5"/>
       <c r="B6" t="s" s="6">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C6" s="7">
         <v>1</v>
       </c>
       <c r="D6" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E6" t="s" s="6">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F6" t="s" s="14">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="G6" t="s" s="15">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="7" ht="13.65" customHeight="1">
       <c r="A7" s="5"/>
       <c r="B7" t="s" s="6">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C7" s="7">
         <v>1</v>
       </c>
       <c r="D7" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E7" t="s" s="6">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F7" t="s" s="14">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="G7" t="s" s="15">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="8" ht="13.65" customHeight="1">
@@ -26789,88 +26818,88 @@
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
       <c r="G8" t="s" s="16">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="9" ht="13.65" customHeight="1">
       <c r="A9" t="s" s="6">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B9" t="s" s="6">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C9" s="7">
         <v>1</v>
       </c>
       <c r="D9" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E9" t="s" s="6">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F9" t="s" s="14">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="G9" t="s" s="15">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="10" ht="13.65" customHeight="1">
       <c r="A10" s="5"/>
       <c r="B10" t="s" s="6">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C10" s="7">
         <v>1</v>
       </c>
       <c r="D10" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E10" t="s" s="6">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F10" t="s" s="14">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="G10" t="s" s="15">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="11" ht="13.65" customHeight="1">
       <c r="A11" s="5"/>
       <c r="B11" t="s" s="6">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C11" s="7">
         <v>1</v>
       </c>
       <c r="D11" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E11" t="s" s="6">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F11" t="s" s="6">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="G11" s="17"/>
     </row>
     <row r="12" ht="13.65" customHeight="1">
       <c r="A12" s="5"/>
       <c r="B12" t="s" s="6">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C12" s="7">
         <v>1</v>
       </c>
       <c r="D12" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E12" t="s" s="6">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F12" t="s" s="6">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="G12" s="5"/>
     </row>
@@ -26885,19 +26914,19 @@
     </row>
     <row r="14" ht="13.65" customHeight="1">
       <c r="A14" t="s" s="6">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B14" t="s" s="6">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C14" s="7">
         <v>1</v>
       </c>
       <c r="D14" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E14" t="s" s="6">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F14" s="5"/>
       <c r="G14" s="5"/>
@@ -26905,16 +26934,16 @@
     <row r="15" ht="13.65" customHeight="1">
       <c r="A15" s="5"/>
       <c r="B15" t="s" s="6">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C15" s="7">
         <v>1</v>
       </c>
       <c r="D15" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E15" t="s" s="6">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F15" s="5"/>
       <c r="G15" s="5"/>
@@ -26922,16 +26951,16 @@
     <row r="16" ht="13.65" customHeight="1">
       <c r="A16" s="5"/>
       <c r="B16" t="s" s="6">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C16" s="7">
         <v>2</v>
       </c>
       <c r="D16" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E16" t="s" s="6">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F16" s="5"/>
       <c r="G16" s="5"/>
@@ -26939,16 +26968,16 @@
     <row r="17" ht="13.65" customHeight="1">
       <c r="A17" s="5"/>
       <c r="B17" t="s" s="6">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C17" s="7">
         <v>2</v>
       </c>
       <c r="D17" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E17" t="s" s="6">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F17" s="5"/>
       <c r="G17" s="5"/>
@@ -26956,16 +26985,16 @@
     <row r="18" ht="13.65" customHeight="1">
       <c r="A18" s="5"/>
       <c r="B18" t="s" s="6">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C18" s="7">
         <v>2</v>
       </c>
       <c r="D18" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E18" t="s" s="6">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F18" s="5"/>
       <c r="G18" s="5"/>
@@ -26973,16 +27002,16 @@
     <row r="19" ht="13.65" customHeight="1">
       <c r="A19" s="5"/>
       <c r="B19" t="s" s="6">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C19" s="7">
         <v>1</v>
       </c>
       <c r="D19" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E19" t="s" s="6">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F19" s="5"/>
       <c r="G19" s="5"/>
@@ -26990,16 +27019,16 @@
     <row r="20" ht="13.65" customHeight="1">
       <c r="A20" s="5"/>
       <c r="B20" t="s" s="6">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C20" s="7">
         <v>1</v>
       </c>
       <c r="D20" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E20" t="s" s="6">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F20" s="5"/>
       <c r="G20" s="5"/>
@@ -27007,16 +27036,16 @@
     <row r="21" ht="13.65" customHeight="1">
       <c r="A21" s="5"/>
       <c r="B21" t="s" s="6">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C21" s="7">
         <v>1</v>
       </c>
       <c r="D21" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E21" t="s" s="6">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F21" s="5"/>
       <c r="G21" s="5"/>
@@ -27024,16 +27053,16 @@
     <row r="22" ht="13.65" customHeight="1">
       <c r="A22" s="5"/>
       <c r="B22" t="s" s="6">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C22" s="7">
         <v>1</v>
       </c>
       <c r="D22" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E22" t="s" s="6">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F22" s="5"/>
       <c r="G22" s="5"/>
@@ -27041,16 +27070,16 @@
     <row r="23" ht="13.65" customHeight="1">
       <c r="A23" s="5"/>
       <c r="B23" t="s" s="6">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C23" s="7">
         <v>1</v>
       </c>
       <c r="D23" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E23" t="s" s="6">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F23" s="5"/>
       <c r="G23" s="5"/>
@@ -27058,16 +27087,16 @@
     <row r="24" ht="13.65" customHeight="1">
       <c r="A24" s="5"/>
       <c r="B24" t="s" s="6">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C24" s="7">
         <v>1</v>
       </c>
       <c r="D24" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E24" t="s" s="6">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F24" s="5"/>
       <c r="G24" s="5"/>
@@ -27083,95 +27112,95 @@
     </row>
     <row r="26" ht="13.65" customHeight="1">
       <c r="A26" t="s" s="6">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B26" t="s" s="6">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C26" s="7">
         <v>1</v>
       </c>
       <c r="D26" t="s" s="6">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E26" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F26" t="s" s="6">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="G26" s="5"/>
     </row>
     <row r="27" ht="13.65" customHeight="1">
       <c r="A27" s="5"/>
       <c r="B27" t="s" s="6">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C27" s="7">
         <v>1</v>
       </c>
       <c r="D27" t="s" s="6">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E27" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F27" t="s" s="6">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="G27" s="5"/>
     </row>
     <row r="28" ht="13.65" customHeight="1">
       <c r="A28" s="5"/>
       <c r="B28" t="s" s="6">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C28" s="7">
         <v>1</v>
       </c>
       <c r="D28" t="s" s="6">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E28" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F28" t="s" s="6">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="G28" s="5"/>
     </row>
     <row r="29" ht="13.65" customHeight="1">
       <c r="A29" s="5"/>
       <c r="B29" t="s" s="6">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C29" s="7">
         <v>1</v>
       </c>
       <c r="D29" t="s" s="6">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E29" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F29" t="s" s="6">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="G29" s="5"/>
     </row>
     <row r="30" ht="13.65" customHeight="1">
       <c r="A30" s="5"/>
       <c r="B30" t="s" s="6">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C30" s="7">
         <v>1</v>
       </c>
       <c r="D30" t="s" s="6">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E30" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F30" s="5"/>
       <c r="G30" s="5"/>
@@ -27179,54 +27208,54 @@
     <row r="31" ht="13.65" customHeight="1">
       <c r="A31" s="5"/>
       <c r="B31" t="s" s="6">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C31" s="7">
         <v>1</v>
       </c>
       <c r="D31" t="s" s="6">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E31" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F31" t="s" s="6">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="G31" s="5"/>
     </row>
     <row r="32" ht="13.65" customHeight="1">
       <c r="A32" s="5"/>
       <c r="B32" t="s" s="6">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C32" s="7">
         <v>1</v>
       </c>
       <c r="D32" t="s" s="6">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E32" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F32" t="s" s="6">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="G32" s="5"/>
     </row>
     <row r="33" ht="13.65" customHeight="1">
       <c r="A33" s="5"/>
       <c r="B33" t="s" s="6">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C33" s="7">
         <v>1</v>
       </c>
       <c r="D33" t="s" s="6">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E33" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F33" s="5"/>
       <c r="G33" s="5"/>
@@ -27234,16 +27263,16 @@
     <row r="34" ht="13.65" customHeight="1">
       <c r="A34" s="5"/>
       <c r="B34" t="s" s="6">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C34" s="7">
         <v>1</v>
       </c>
       <c r="D34" t="s" s="6">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E34" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F34" s="5"/>
       <c r="G34" s="5"/>
@@ -27251,16 +27280,16 @@
     <row r="35" ht="13.65" customHeight="1">
       <c r="A35" s="5"/>
       <c r="B35" t="s" s="6">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C35" s="7">
         <v>1</v>
       </c>
       <c r="D35" t="s" s="6">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E35" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F35" s="5"/>
       <c r="G35" s="5"/>
@@ -27268,16 +27297,16 @@
     <row r="36" ht="13.65" customHeight="1">
       <c r="A36" s="5"/>
       <c r="B36" t="s" s="6">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C36" s="7">
         <v>1</v>
       </c>
       <c r="D36" t="s" s="6">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E36" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F36" s="5"/>
       <c r="G36" s="5"/>
@@ -27285,16 +27314,16 @@
     <row r="37" ht="13.65" customHeight="1">
       <c r="A37" s="5"/>
       <c r="B37" t="s" s="6">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C37" s="7">
         <v>1</v>
       </c>
       <c r="D37" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E37" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F37" s="5"/>
       <c r="G37" s="5"/>
@@ -27302,16 +27331,16 @@
     <row r="38" ht="13.65" customHeight="1">
       <c r="A38" s="5"/>
       <c r="B38" t="s" s="6">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C38" s="7">
         <v>1</v>
       </c>
       <c r="D38" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E38" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F38" s="5"/>
       <c r="G38" s="5"/>
@@ -27319,16 +27348,16 @@
     <row r="39" ht="13.65" customHeight="1">
       <c r="A39" s="5"/>
       <c r="B39" t="s" s="6">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C39" s="7">
         <v>1</v>
       </c>
       <c r="D39" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E39" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F39" s="5"/>
       <c r="G39" s="5"/>
@@ -27336,16 +27365,16 @@
     <row r="40" ht="13.65" customHeight="1">
       <c r="A40" s="5"/>
       <c r="B40" t="s" s="6">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C40" s="7">
         <v>1</v>
       </c>
       <c r="D40" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E40" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F40" s="5"/>
       <c r="G40" s="5"/>
@@ -27353,16 +27382,16 @@
     <row r="41" ht="13.65" customHeight="1">
       <c r="A41" s="5"/>
       <c r="B41" t="s" s="6">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C41" s="7">
         <v>2</v>
       </c>
       <c r="D41" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E41" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F41" s="5"/>
       <c r="G41" s="5"/>
@@ -27370,111 +27399,111 @@
     <row r="42" ht="13.65" customHeight="1">
       <c r="A42" s="5"/>
       <c r="B42" t="s" s="6">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C42" s="7">
         <v>1</v>
       </c>
       <c r="D42" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E42" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F42" t="s" s="6">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="G42" s="5"/>
     </row>
     <row r="43" ht="13.65" customHeight="1">
       <c r="A43" s="5"/>
       <c r="B43" t="s" s="6">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C43" s="7">
         <v>1</v>
       </c>
       <c r="D43" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E43" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F43" t="s" s="6">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="G43" s="5"/>
     </row>
     <row r="44" ht="13.65" customHeight="1">
       <c r="A44" s="5"/>
       <c r="B44" t="s" s="6">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C44" s="7">
         <v>1</v>
       </c>
       <c r="D44" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E44" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F44" t="s" s="6">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="G44" s="5"/>
     </row>
     <row r="45" ht="13.65" customHeight="1">
       <c r="A45" s="5"/>
       <c r="B45" t="s" s="6">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C45" s="7">
         <v>1</v>
       </c>
       <c r="D45" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E45" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F45" t="s" s="6">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="G45" s="5"/>
     </row>
     <row r="46" ht="13.65" customHeight="1">
       <c r="A46" s="5"/>
       <c r="B46" t="s" s="6">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C46" s="7">
         <v>1</v>
       </c>
       <c r="D46" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E46" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F46" t="s" s="6">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="G46" s="5"/>
     </row>
     <row r="47" ht="13.65" customHeight="1">
       <c r="A47" s="5"/>
       <c r="B47" t="s" s="6">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C47" s="7">
         <v>1</v>
       </c>
       <c r="D47" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E47" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F47" s="5"/>
       <c r="G47" s="5"/>
@@ -27482,16 +27511,16 @@
     <row r="48" ht="13.65" customHeight="1">
       <c r="A48" s="5"/>
       <c r="B48" t="s" s="6">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C48" s="7">
         <v>1</v>
       </c>
       <c r="D48" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E48" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F48" s="5"/>
       <c r="G48" s="5"/>
@@ -27499,16 +27528,16 @@
     <row r="49" ht="13.65" customHeight="1">
       <c r="A49" s="5"/>
       <c r="B49" t="s" s="6">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C49" s="7">
         <v>1</v>
       </c>
       <c r="D49" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E49" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F49" s="5"/>
       <c r="G49" s="5"/>
@@ -27516,54 +27545,54 @@
     <row r="50" ht="13.65" customHeight="1">
       <c r="A50" s="5"/>
       <c r="B50" t="s" s="6">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C50" s="7">
         <v>1</v>
       </c>
       <c r="D50" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E50" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F50" t="s" s="6">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="G50" s="5"/>
     </row>
     <row r="51" ht="13.65" customHeight="1">
       <c r="A51" s="5"/>
       <c r="B51" t="s" s="6">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C51" s="7">
         <v>1</v>
       </c>
       <c r="D51" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E51" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F51" t="s" s="6">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="G51" s="5"/>
     </row>
     <row r="52" ht="13.65" customHeight="1">
       <c r="A52" s="5"/>
       <c r="B52" t="s" s="6">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C52" s="7">
         <v>1</v>
       </c>
       <c r="D52" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E52" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F52" s="5"/>
       <c r="G52" s="5"/>
@@ -27571,16 +27600,16 @@
     <row r="53" ht="13.65" customHeight="1">
       <c r="A53" s="5"/>
       <c r="B53" t="s" s="6">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C53" s="7">
         <v>1</v>
       </c>
       <c r="D53" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E53" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F53" s="5"/>
       <c r="G53" s="5"/>
@@ -27596,19 +27625,19 @@
     </row>
     <row r="55" ht="13.65" customHeight="1">
       <c r="A55" t="s" s="6">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B55" t="s" s="6">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C55" s="7">
         <v>1</v>
       </c>
       <c r="D55" t="s" s="6">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E55" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F55" s="5"/>
       <c r="G55" s="5"/>
@@ -27616,16 +27645,16 @@
     <row r="56" ht="13.65" customHeight="1">
       <c r="A56" s="5"/>
       <c r="B56" t="s" s="6">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C56" s="7">
         <v>1</v>
       </c>
       <c r="D56" t="s" s="6">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E56" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F56" s="5"/>
       <c r="G56" s="5"/>
@@ -27633,16 +27662,16 @@
     <row r="57" ht="13.65" customHeight="1">
       <c r="A57" s="5"/>
       <c r="B57" t="s" s="6">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C57" s="7">
         <v>1</v>
       </c>
       <c r="D57" t="s" s="6">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E57" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F57" s="5"/>
       <c r="G57" s="5"/>
@@ -27650,16 +27679,16 @@
     <row r="58" ht="13.65" customHeight="1">
       <c r="A58" s="5"/>
       <c r="B58" t="s" s="6">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C58" s="7">
         <v>1</v>
       </c>
       <c r="D58" t="s" s="6">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E58" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F58" s="5"/>
       <c r="G58" s="5"/>
@@ -27667,16 +27696,16 @@
     <row r="59" ht="13.65" customHeight="1">
       <c r="A59" s="5"/>
       <c r="B59" t="s" s="6">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C59" s="7">
         <v>2</v>
       </c>
       <c r="D59" t="s" s="6">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E59" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F59" s="5"/>
       <c r="G59" s="5"/>
@@ -27684,16 +27713,16 @@
     <row r="60" ht="13.65" customHeight="1">
       <c r="A60" s="5"/>
       <c r="B60" t="s" s="6">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C60" s="7">
         <v>1</v>
       </c>
       <c r="D60" t="s" s="6">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="E60" t="s" s="6">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="F60" s="5"/>
       <c r="G60" s="5"/>
@@ -27701,16 +27730,16 @@
     <row r="61" ht="13.65" customHeight="1">
       <c r="A61" s="5"/>
       <c r="B61" t="s" s="6">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C61" s="7">
         <v>1</v>
       </c>
       <c r="D61" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E61" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F61" s="5"/>
       <c r="G61" s="5"/>
@@ -27718,16 +27747,16 @@
     <row r="62" ht="13.65" customHeight="1">
       <c r="A62" s="5"/>
       <c r="B62" t="s" s="6">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C62" s="7">
         <v>2</v>
       </c>
       <c r="D62" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E62" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F62" s="5"/>
       <c r="G62" s="5"/>
@@ -27735,16 +27764,16 @@
     <row r="63" ht="13.65" customHeight="1">
       <c r="A63" s="5"/>
       <c r="B63" t="s" s="6">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C63" s="7">
         <v>1</v>
       </c>
       <c r="D63" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E63" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F63" s="5"/>
       <c r="G63" s="5"/>
@@ -27752,16 +27781,16 @@
     <row r="64" ht="13.65" customHeight="1">
       <c r="A64" s="5"/>
       <c r="B64" t="s" s="6">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C64" s="7">
         <v>2</v>
       </c>
       <c r="D64" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E64" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F64" s="5"/>
       <c r="G64" s="5"/>
@@ -27769,16 +27798,16 @@
     <row r="65" ht="13.65" customHeight="1">
       <c r="A65" s="5"/>
       <c r="B65" t="s" s="6">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C65" s="7">
         <v>8</v>
       </c>
       <c r="D65" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E65" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F65" s="5"/>
       <c r="G65" s="5"/>
@@ -27786,111 +27815,111 @@
     <row r="66" ht="13.65" customHeight="1">
       <c r="A66" s="5"/>
       <c r="B66" t="s" s="6">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C66" s="7">
         <v>1</v>
       </c>
       <c r="D66" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E66" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F66" t="s" s="6">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="G66" s="5"/>
     </row>
     <row r="67" ht="13.65" customHeight="1">
       <c r="A67" s="5"/>
       <c r="B67" t="s" s="6">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C67" s="7">
         <v>1</v>
       </c>
       <c r="D67" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E67" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F67" t="s" s="6">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="G67" s="5"/>
     </row>
     <row r="68" ht="13.65" customHeight="1">
       <c r="A68" s="5"/>
       <c r="B68" t="s" s="6">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C68" s="7">
         <v>2</v>
       </c>
       <c r="D68" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E68" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F68" t="s" s="6">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="G68" s="5"/>
     </row>
     <row r="69" ht="13.65" customHeight="1">
       <c r="A69" s="5"/>
       <c r="B69" t="s" s="6">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C69" s="7">
         <v>1</v>
       </c>
       <c r="D69" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E69" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F69" t="s" s="6">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="G69" s="5"/>
     </row>
     <row r="70" ht="13.65" customHeight="1">
       <c r="A70" s="5"/>
       <c r="B70" t="s" s="6">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C70" s="7">
         <v>1</v>
       </c>
       <c r="D70" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E70" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F70" t="s" s="6">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="G70" s="5"/>
     </row>
     <row r="71" ht="13.65" customHeight="1">
       <c r="A71" s="5"/>
       <c r="B71" t="s" s="6">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C71" s="7">
         <v>1</v>
       </c>
       <c r="D71" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E71" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F71" s="5"/>
       <c r="G71" s="5"/>
@@ -27898,16 +27927,16 @@
     <row r="72" ht="13.65" customHeight="1">
       <c r="A72" s="5"/>
       <c r="B72" t="s" s="6">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C72" s="7">
         <v>1</v>
       </c>
       <c r="D72" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E72" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F72" s="5"/>
       <c r="G72" s="5"/>
@@ -27915,16 +27944,16 @@
     <row r="73" ht="13.65" customHeight="1">
       <c r="A73" s="5"/>
       <c r="B73" t="s" s="6">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C73" s="7">
         <v>1</v>
       </c>
       <c r="D73" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E73" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F73" s="5"/>
       <c r="G73" s="5"/>
@@ -27940,19 +27969,19 @@
     </row>
     <row r="75" ht="13.65" customHeight="1">
       <c r="A75" t="s" s="6">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B75" t="s" s="6">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C75" s="7">
         <v>6</v>
       </c>
       <c r="D75" t="s" s="6">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E75" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F75" s="5"/>
       <c r="G75" s="5"/>
@@ -27960,16 +27989,16 @@
     <row r="76" ht="13.65" customHeight="1">
       <c r="A76" s="5"/>
       <c r="B76" t="s" s="6">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C76" s="7">
         <v>4</v>
       </c>
       <c r="D76" t="s" s="6">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E76" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F76" s="5"/>
       <c r="G76" s="5"/>
@@ -27977,16 +28006,16 @@
     <row r="77" ht="13.65" customHeight="1">
       <c r="A77" s="5"/>
       <c r="B77" t="s" s="6">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C77" s="7">
         <v>3</v>
       </c>
       <c r="D77" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E77" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F77" s="5"/>
       <c r="G77" s="5"/>
@@ -27994,16 +28023,16 @@
     <row r="78" ht="13.65" customHeight="1">
       <c r="A78" s="5"/>
       <c r="B78" t="s" s="6">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C78" s="7">
         <v>1</v>
       </c>
       <c r="D78" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E78" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F78" s="5"/>
       <c r="G78" s="5"/>
@@ -28011,16 +28040,16 @@
     <row r="79" ht="13.65" customHeight="1">
       <c r="A79" s="5"/>
       <c r="B79" t="s" s="6">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C79" s="7">
         <v>1</v>
       </c>
       <c r="D79" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E79" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F79" s="5"/>
       <c r="G79" s="5"/>
@@ -28028,16 +28057,16 @@
     <row r="80" ht="13.65" customHeight="1">
       <c r="A80" s="5"/>
       <c r="B80" t="s" s="6">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C80" s="7">
         <v>1</v>
       </c>
       <c r="D80" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E80" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F80" s="5"/>
       <c r="G80" s="5"/>
@@ -28053,19 +28082,19 @@
     </row>
     <row r="82" ht="13.65" customHeight="1">
       <c r="A82" t="s" s="6">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B82" t="s" s="6">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C82" s="7">
         <v>2</v>
       </c>
       <c r="D82" t="s" s="6">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E82" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F82" s="5"/>
       <c r="G82" s="5"/>
@@ -28073,16 +28102,16 @@
     <row r="83" ht="13.65" customHeight="1">
       <c r="A83" s="5"/>
       <c r="B83" t="s" s="6">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C83" s="7">
         <v>2</v>
       </c>
       <c r="D83" t="s" s="6">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E83" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F83" s="5"/>
       <c r="G83" s="5"/>
@@ -28090,16 +28119,16 @@
     <row r="84" ht="13.65" customHeight="1">
       <c r="A84" s="5"/>
       <c r="B84" t="s" s="6">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C84" s="7">
         <v>1</v>
       </c>
       <c r="D84" t="s" s="6">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E84" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F84" s="5"/>
       <c r="G84" s="5"/>
@@ -28107,16 +28136,16 @@
     <row r="85" ht="13.65" customHeight="1">
       <c r="A85" s="5"/>
       <c r="B85" t="s" s="6">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C85" s="7">
         <v>1</v>
       </c>
       <c r="D85" t="s" s="6">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E85" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F85" s="5"/>
       <c r="G85" s="5"/>
@@ -28124,16 +28153,16 @@
     <row r="86" ht="13.65" customHeight="1">
       <c r="A86" s="5"/>
       <c r="B86" t="s" s="6">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C86" s="7">
         <v>1</v>
       </c>
       <c r="D86" t="s" s="6">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E86" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F86" s="5"/>
       <c r="G86" s="5"/>
@@ -28141,16 +28170,16 @@
     <row r="87" ht="13.65" customHeight="1">
       <c r="A87" s="5"/>
       <c r="B87" t="s" s="6">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C87" s="7">
         <v>1</v>
       </c>
       <c r="D87" t="s" s="6">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E87" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F87" s="5"/>
       <c r="G87" s="5"/>
@@ -28158,16 +28187,16 @@
     <row r="88" ht="13.65" customHeight="1">
       <c r="A88" s="5"/>
       <c r="B88" t="s" s="6">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C88" s="7">
         <v>1</v>
       </c>
       <c r="D88" t="s" s="6">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E88" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F88" s="5"/>
       <c r="G88" s="5"/>
@@ -28175,16 +28204,16 @@
     <row r="89" ht="13.65" customHeight="1">
       <c r="A89" s="5"/>
       <c r="B89" t="s" s="6">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C89" s="7">
         <v>1</v>
       </c>
       <c r="D89" t="s" s="6">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E89" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F89" s="5"/>
       <c r="G89" s="5"/>
@@ -28192,16 +28221,16 @@
     <row r="90" ht="13.65" customHeight="1">
       <c r="A90" s="5"/>
       <c r="B90" t="s" s="6">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C90" s="7">
         <v>1</v>
       </c>
       <c r="D90" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E90" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F90" s="5"/>
       <c r="G90" s="5"/>
@@ -28209,16 +28238,16 @@
     <row r="91" ht="13.65" customHeight="1">
       <c r="A91" s="5"/>
       <c r="B91" t="s" s="6">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C91" s="7">
         <v>1</v>
       </c>
       <c r="D91" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E91" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F91" s="5"/>
       <c r="G91" s="5"/>
@@ -28226,76 +28255,76 @@
     <row r="92" ht="13.65" customHeight="1">
       <c r="A92" s="5"/>
       <c r="B92" t="s" s="6">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C92" s="7">
         <v>1</v>
       </c>
       <c r="D92" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E92" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F92" t="s" s="6">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="G92" s="5"/>
     </row>
     <row r="93" ht="13.65" customHeight="1">
       <c r="A93" s="5"/>
       <c r="B93" t="s" s="6">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C93" s="7">
         <v>1</v>
       </c>
       <c r="D93" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E93" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F93" t="s" s="6">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="G93" s="5"/>
     </row>
     <row r="94" ht="13.65" customHeight="1">
       <c r="A94" s="5"/>
       <c r="B94" t="s" s="6">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C94" s="7">
         <v>1</v>
       </c>
       <c r="D94" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E94" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F94" t="s" s="6">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="G94" s="5"/>
     </row>
     <row r="95" ht="13.65" customHeight="1">
       <c r="A95" s="5"/>
       <c r="B95" t="s" s="6">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C95" s="7">
         <v>1</v>
       </c>
       <c r="D95" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E95" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F95" t="s" s="6">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="G95" s="5"/>
     </row>
@@ -28310,19 +28339,19 @@
     </row>
     <row r="97" ht="13.65" customHeight="1">
       <c r="A97" t="s" s="6">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="B97" t="s" s="6">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C97" s="7">
         <v>1</v>
       </c>
       <c r="D97" t="s" s="6">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E97" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F97" s="5"/>
       <c r="G97" s="5"/>
@@ -28330,16 +28359,16 @@
     <row r="98" ht="13.65" customHeight="1">
       <c r="A98" s="5"/>
       <c r="B98" t="s" s="6">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C98" s="7">
         <v>2</v>
       </c>
       <c r="D98" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E98" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F98" s="5"/>
       <c r="G98" s="5"/>
@@ -28347,16 +28376,16 @@
     <row r="99" ht="13.65" customHeight="1">
       <c r="A99" s="5"/>
       <c r="B99" t="s" s="6">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="C99" s="7">
         <v>2</v>
       </c>
       <c r="D99" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E99" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F99" s="5"/>
       <c r="G99" s="5"/>
@@ -28364,16 +28393,16 @@
     <row r="100" ht="13.65" customHeight="1">
       <c r="A100" s="5"/>
       <c r="B100" t="s" s="6">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C100" s="7">
         <v>1</v>
       </c>
       <c r="D100" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E100" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F100" s="5"/>
       <c r="G100" s="5"/>
@@ -28381,16 +28410,16 @@
     <row r="101" ht="13.65" customHeight="1">
       <c r="A101" s="5"/>
       <c r="B101" t="s" s="6">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C101" s="7">
         <v>1</v>
       </c>
       <c r="D101" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E101" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F101" s="5"/>
       <c r="G101" s="5"/>
@@ -28398,16 +28427,16 @@
     <row r="102" ht="13.65" customHeight="1">
       <c r="A102" s="5"/>
       <c r="B102" t="s" s="6">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C102" s="7">
         <v>1</v>
       </c>
       <c r="D102" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E102" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F102" s="5"/>
       <c r="G102" s="5"/>
@@ -28415,16 +28444,16 @@
     <row r="103" ht="13.65" customHeight="1">
       <c r="A103" s="5"/>
       <c r="B103" t="s" s="6">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="C103" s="7">
         <v>1</v>
       </c>
       <c r="D103" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E103" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F103" s="5"/>
       <c r="G103" s="5"/>
@@ -28432,16 +28461,16 @@
     <row r="104" ht="13.65" customHeight="1">
       <c r="A104" s="5"/>
       <c r="B104" t="s" s="6">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C104" s="7">
         <v>2</v>
       </c>
       <c r="D104" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E104" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F104" s="5"/>
       <c r="G104" s="5"/>
@@ -28449,16 +28478,16 @@
     <row r="105" ht="13.65" customHeight="1">
       <c r="A105" s="5"/>
       <c r="B105" t="s" s="6">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="C105" s="7">
         <v>1</v>
       </c>
       <c r="D105" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E105" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F105" s="5"/>
       <c r="G105" s="5"/>
@@ -28466,16 +28495,16 @@
     <row r="106" ht="13.65" customHeight="1">
       <c r="A106" s="5"/>
       <c r="B106" t="s" s="6">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C106" s="7">
         <v>1</v>
       </c>
       <c r="D106" t="s" s="6">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E106" t="s" s="6">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F106" s="5"/>
       <c r="G106" s="5"/>
@@ -28491,7 +28520,7 @@
     </row>
     <row r="108" ht="13.65" customHeight="1">
       <c r="A108" t="s" s="2">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="B108" s="5"/>
       <c r="C108" s="5"/>
@@ -28502,19 +28531,19 @@
     </row>
     <row r="109" ht="13.65" customHeight="1">
       <c r="A109" t="s" s="6">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B109" t="s" s="6">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="C109" s="7">
         <v>1</v>
       </c>
       <c r="D109" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E109" t="s" s="6">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="F109" s="5"/>
       <c r="G109" s="5"/>
@@ -28522,16 +28551,16 @@
     <row r="110" ht="13.65" customHeight="1">
       <c r="A110" s="5"/>
       <c r="B110" t="s" s="6">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="C110" s="7">
         <v>1</v>
       </c>
       <c r="D110" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E110" t="s" s="6">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="F110" s="5"/>
       <c r="G110" s="5"/>
@@ -28539,16 +28568,16 @@
     <row r="111" ht="13.65" customHeight="1">
       <c r="A111" s="5"/>
       <c r="B111" t="s" s="6">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C111" s="7">
         <v>1</v>
       </c>
       <c r="D111" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E111" t="s" s="6">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="F111" s="5"/>
       <c r="G111" s="5"/>
@@ -28556,16 +28585,16 @@
     <row r="112" ht="13.65" customHeight="1">
       <c r="A112" s="5"/>
       <c r="B112" t="s" s="6">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="C112" s="7">
         <v>1</v>
       </c>
       <c r="D112" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E112" t="s" s="6">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="F112" s="5"/>
       <c r="G112" s="5"/>
@@ -28573,16 +28602,16 @@
     <row r="113" ht="13.65" customHeight="1">
       <c r="A113" s="5"/>
       <c r="B113" t="s" s="6">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="C113" s="7">
         <v>2</v>
       </c>
       <c r="D113" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E113" t="s" s="6">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="F113" s="5"/>
       <c r="G113" s="5"/>
@@ -28590,16 +28619,16 @@
     <row r="114" ht="13.65" customHeight="1">
       <c r="A114" s="5"/>
       <c r="B114" t="s" s="6">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="C114" s="7">
         <v>1</v>
       </c>
       <c r="D114" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E114" t="s" s="6">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="F114" s="5"/>
       <c r="G114" s="5"/>
@@ -28607,76 +28636,76 @@
     <row r="115" ht="13.65" customHeight="1">
       <c r="A115" s="5"/>
       <c r="B115" t="s" s="6">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="C115" s="7">
         <v>1</v>
       </c>
       <c r="D115" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E115" t="s" s="6">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="F115" t="s" s="6">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="G115" s="5"/>
     </row>
     <row r="116" ht="13.65" customHeight="1">
       <c r="A116" s="5"/>
       <c r="B116" t="s" s="6">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="C116" s="7">
         <v>1</v>
       </c>
       <c r="D116" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E116" t="s" s="6">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="F116" t="s" s="6">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="G116" s="5"/>
     </row>
     <row r="117" ht="13.65" customHeight="1">
       <c r="A117" s="5"/>
       <c r="B117" t="s" s="6">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="C117" s="7">
         <v>1</v>
       </c>
       <c r="D117" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E117" t="s" s="6">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="F117" t="s" s="6">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="G117" s="5"/>
     </row>
     <row r="118" ht="13.65" customHeight="1">
       <c r="A118" s="5"/>
       <c r="B118" t="s" s="6">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C118" s="7">
         <v>1</v>
       </c>
       <c r="D118" t="s" s="6">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E118" t="s" s="6">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="F118" t="s" s="6">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="G118" s="5"/>
     </row>
@@ -28691,7 +28720,7 @@
     </row>
     <row r="120" ht="13.65" customHeight="1">
       <c r="A120" t="s" s="2">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B120" s="5"/>
       <c r="C120" s="5"/>
@@ -28702,88 +28731,88 @@
     </row>
     <row r="121" ht="13.65" customHeight="1">
       <c r="A121" t="s" s="6">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B121" t="s" s="6">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="C121" s="7">
         <v>1</v>
       </c>
       <c r="D121" s="5"/>
       <c r="E121" t="s" s="6">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="F121" t="s" s="6">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="G121" s="5"/>
     </row>
     <row r="122" ht="13.65" customHeight="1">
       <c r="A122" s="5"/>
       <c r="B122" t="s" s="6">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C122" s="7">
         <v>1</v>
       </c>
       <c r="D122" s="5"/>
       <c r="E122" t="s" s="6">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="F122" t="s" s="6">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="G122" s="5"/>
     </row>
     <row r="123" ht="13.65" customHeight="1">
       <c r="A123" s="5"/>
       <c r="B123" t="s" s="6">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="C123" s="7">
         <v>2</v>
       </c>
       <c r="D123" s="5"/>
       <c r="E123" t="s" s="6">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="F123" t="s" s="6">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="G123" s="5"/>
     </row>
     <row r="124" ht="13.65" customHeight="1">
       <c r="A124" s="5"/>
       <c r="B124" t="s" s="6">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="C124" s="7">
         <v>1</v>
       </c>
       <c r="D124" s="5"/>
       <c r="E124" t="s" s="6">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="F124" t="s" s="6">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="G124" s="5"/>
     </row>
     <row r="125" ht="13.65" customHeight="1">
       <c r="A125" s="5"/>
       <c r="B125" t="s" s="6">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C125" s="7">
         <v>1</v>
       </c>
       <c r="D125" s="5"/>
       <c r="E125" t="s" s="6">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="F125" t="s" s="6">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="G125" s="5"/>
     </row>
@@ -28798,71 +28827,71 @@
     </row>
     <row r="127" ht="13.65" customHeight="1">
       <c r="A127" t="s" s="6">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B127" t="s" s="6">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C127" s="7">
         <v>1</v>
       </c>
       <c r="D127" s="5"/>
       <c r="E127" t="s" s="6">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="F127" t="s" s="6">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="G127" s="5"/>
     </row>
     <row r="128" ht="13.65" customHeight="1">
       <c r="A128" s="5"/>
       <c r="B128" t="s" s="6">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C128" s="7">
         <v>1</v>
       </c>
       <c r="D128" s="5"/>
       <c r="E128" t="s" s="6">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="F128" t="s" s="6">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="G128" s="5"/>
     </row>
     <row r="129" ht="13.65" customHeight="1">
       <c r="A129" s="5"/>
       <c r="B129" t="s" s="6">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="C129" s="7">
         <v>1</v>
       </c>
       <c r="D129" s="5"/>
       <c r="E129" t="s" s="6">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="F129" t="s" s="6">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="G129" s="5"/>
     </row>
     <row r="130" ht="13.65" customHeight="1">
       <c r="A130" s="5"/>
       <c r="B130" t="s" s="6">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C130" s="7">
         <v>2</v>
       </c>
       <c r="D130" s="5"/>
       <c r="E130" t="s" s="6">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="F130" t="s" s="6">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="G130" s="5"/>
     </row>
@@ -28877,90 +28906,90 @@
     </row>
     <row r="132" ht="13.65" customHeight="1">
       <c r="A132" t="s" s="6">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B132" t="s" s="6">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C132" s="7">
         <v>1</v>
       </c>
       <c r="D132" s="5"/>
       <c r="E132" t="s" s="6">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="F132" t="s" s="6">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="G132" s="5"/>
     </row>
     <row r="133" ht="13.65" customHeight="1">
       <c r="A133" t="s" s="6">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="B133" t="s" s="6">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="C133" s="7">
         <v>1</v>
       </c>
       <c r="D133" s="5"/>
       <c r="E133" t="s" s="6">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="F133" t="s" s="6">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="G133" s="5"/>
     </row>
     <row r="134" ht="13.65" customHeight="1">
       <c r="A134" s="5"/>
       <c r="B134" t="s" s="6">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="C134" s="7">
         <v>1</v>
       </c>
       <c r="D134" s="5"/>
       <c r="E134" t="s" s="6">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="F134" t="s" s="6">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="G134" s="5"/>
     </row>
     <row r="135" ht="13.65" customHeight="1">
       <c r="A135" s="5"/>
       <c r="B135" t="s" s="6">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="C135" s="7">
         <v>1</v>
       </c>
       <c r="D135" s="5"/>
       <c r="E135" t="s" s="6">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="F135" t="s" s="6">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="G135" s="5"/>
     </row>
     <row r="136" ht="13.65" customHeight="1">
       <c r="A136" s="5"/>
       <c r="B136" t="s" s="6">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C136" s="7">
         <v>1</v>
       </c>
       <c r="D136" s="5"/>
       <c r="E136" t="s" s="6">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="F136" t="s" s="6">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="G136" s="5"/>
     </row>
@@ -29260,7 +29289,7 @@
   <sheetData>
     <row r="1" ht="13.65" customHeight="1">
       <c r="A1" t="s" s="19">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -29285,7 +29314,7 @@
     </row>
     <row r="2" ht="13.65" customHeight="1">
       <c r="A2" t="s" s="20">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
@@ -29333,16 +29362,16 @@
     </row>
     <row r="4" ht="13.65" customHeight="1">
       <c r="A4" t="s" s="4">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B4" t="s" s="4">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C4" t="s" s="4">
         <v>2</v>
       </c>
       <c r="D4" t="s" s="4">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="E4" s="8"/>
       <c r="F4" s="8"/>
@@ -29364,7 +29393,7 @@
     </row>
     <row r="5" ht="13.65" customHeight="1">
       <c r="A5" t="s" s="6">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="7">
@@ -29391,7 +29420,7 @@
     </row>
     <row r="6" ht="13.65" customHeight="1">
       <c r="A6" t="s" s="6">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="7">
@@ -29418,14 +29447,14 @@
     </row>
     <row r="7" ht="13.65" customHeight="1">
       <c r="A7" t="s" s="6">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="7">
         <v>1</v>
       </c>
       <c r="D7" t="s" s="21">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
@@ -29447,7 +29476,7 @@
     </row>
     <row r="8" ht="13.65" customHeight="1">
       <c r="A8" t="s" s="6">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B8" s="5"/>
       <c r="C8" s="7">
@@ -29474,7 +29503,7 @@
     </row>
     <row r="9" ht="13.65" customHeight="1">
       <c r="A9" t="s" s="6">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="B9" s="5"/>
       <c r="C9" s="7">
@@ -29501,10 +29530,10 @@
     </row>
     <row r="10" ht="13.65" customHeight="1">
       <c r="A10" t="s" s="6">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="B10" t="s" s="6">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="C10" s="7">
         <v>1</v>
@@ -29530,10 +29559,10 @@
     </row>
     <row r="11" ht="13.65" customHeight="1">
       <c r="A11" t="s" s="6">
+        <v>473</v>
+      </c>
+      <c r="B11" t="s" s="6">
         <v>472</v>
-      </c>
-      <c r="B11" t="s" s="6">
-        <v>471</v>
       </c>
       <c r="C11" s="7">
         <v>1</v>
@@ -29559,7 +29588,7 @@
     </row>
     <row r="12" ht="13.65" customHeight="1">
       <c r="A12" t="s" s="6">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="7">
@@ -29586,7 +29615,7 @@
     </row>
     <row r="13" ht="13.65" customHeight="1">
       <c r="A13" t="s" s="6">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B13" s="5"/>
       <c r="C13" s="7">
@@ -29613,7 +29642,7 @@
     </row>
     <row r="14" ht="13.65" customHeight="1">
       <c r="A14" t="s" s="6">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B14" s="5"/>
       <c r="C14" s="7">
@@ -29640,7 +29669,7 @@
     </row>
     <row r="15" ht="13.65" customHeight="1">
       <c r="A15" t="s" s="6">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B15" s="5"/>
       <c r="C15" s="7">
@@ -29713,7 +29742,7 @@
     </row>
     <row r="18" ht="13.65" customHeight="1">
       <c r="A18" t="s" s="4">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -29738,7 +29767,7 @@
     </row>
     <row r="19" ht="13.65" customHeight="1">
       <c r="A19" t="s" s="6">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="7">
@@ -29765,10 +29794,10 @@
     </row>
     <row r="20" ht="13.65" customHeight="1">
       <c r="A20" t="s" s="6">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="B20" t="s" s="6">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="C20" s="7">
         <v>4</v>
@@ -29794,7 +29823,7 @@
     </row>
     <row r="21" ht="13.65" customHeight="1">
       <c r="A21" t="s" s="6">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="7">
@@ -29821,7 +29850,7 @@
     </row>
     <row r="22" ht="13.65" customHeight="1">
       <c r="A22" t="s" s="6">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="7">

</xml_diff>